<commit_message>
Se cargan archivos 16_04_2026 sin zip
</commit_message>
<xml_diff>
--- a/DataSphere/Encuestas Satisfaccion/2020 ajuste campos.xlsx
+++ b/DataSphere/Encuestas Satisfaccion/2020 ajuste campos.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\degonzalez\Documents\2026\Backup_2026\DataSphere\Encuestas Satisfaccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD235F94-F681-4F38-B49F-10C6ACF052BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5109EE-B8E0-4089-8BA2-F9D104BCF4CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{30568307-A7DA-4B3B-8791-30F5B1CB29BF}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{30568307-A7DA-4B3B-8791-30F5B1CB29BF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="2020" sheetId="1" r:id="rId1"/>
+    <sheet name="2019" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="81">
   <si>
     <t>NULL As "Tipo_Formacion",</t>
   </si>
@@ -150,6 +151,138 @@
   </si>
   <si>
     <t>"Year" As Año</t>
+  </si>
+  <si>
+    <t>"ID_2019" AS "Año"</t>
+  </si>
+  <si>
+    <t>NULL As "Facultad",</t>
+  </si>
+  <si>
+    <t>"cedula" As "Cedula",</t>
+  </si>
+  <si>
+    <t>"Modalidad" As "Metododologia",</t>
+  </si>
+  <si>
+    <t>Para iniciar, por favor, indícanos el número de tu documento de identidad: As "Documento_identidad",</t>
+  </si>
+  <si>
+    <t>Modalidad As "Modalidad",</t>
+  </si>
+  <si>
+    <t>Tipo de Formación  As "Tipo_Formacion",</t>
+  </si>
+  <si>
+    <t>ACA1 As "Plan de estudios de tu programa",</t>
+  </si>
+  <si>
+    <t>ACA2 As "Pertinencia de los conocimientos adquiridos en las clases",</t>
+  </si>
+  <si>
+    <t>ACA3 As "Contribución del programa en tu proceso formativo",</t>
+  </si>
+  <si>
+    <t>ACA4 As "¿Qué tan cumplida ha sido la Universidad Ean respecto a la promesa de valor académica ofrecida por el programa que cursas actualmente?",</t>
+  </si>
+  <si>
+    <t>ACA5 As "Conforme al avance de tu programa académico:",</t>
+  </si>
+  <si>
+    <t>ACA6 As "Conocimiento disciplinar",</t>
+  </si>
+  <si>
+    <t>ACA7 As "Competencias para la enseñanza y la formación",</t>
+  </si>
+  <si>
+    <t>ACA8 As "Cumplimiento del syllabus y plan de estudios del programa",</t>
+  </si>
+  <si>
+    <t>ACA9 As "Evaluación y acompañamiento del proceso de aprendizaje",</t>
+  </si>
+  <si>
+    <t>ACA10 As "Entrega de calificaciones y retroalimentación",</t>
+  </si>
+  <si>
+    <t>ACA11 As "Calidad humana",</t>
+  </si>
+  <si>
+    <t>ACA12 As "Compromiso",</t>
+  </si>
+  <si>
+    <t>ACA13 As "Manejo tecnológico",</t>
+  </si>
+  <si>
+    <t>ACA14 As "Decano(a)",</t>
+  </si>
+  <si>
+    <t>ACA15 As "Director(a) de Programa o Coordinador",</t>
+  </si>
+  <si>
+    <t>ACA16 As "Satisfacción entrega material VAC",</t>
+  </si>
+  <si>
+    <t>ACA17 As "Satisfacción asistentes facultad",</t>
+  </si>
+  <si>
+    <t>ACA18 As "Probabilidad recomendar programa académico",</t>
+  </si>
+  <si>
+    <t>ACA19 As "Probabilidad volver a estudiar en EAN",</t>
+  </si>
+  <si>
+    <t>ACA20 As "Cuerpo docente con experiencia profesional"</t>
+  </si>
+  <si>
+    <t>NULL As "Programa",</t>
+  </si>
+  <si>
+    <t>"AC1" As "Plan de estudios de tu programa",</t>
+  </si>
+  <si>
+    <t>NULL  As "Conocimiento disciplinar",</t>
+  </si>
+  <si>
+    <t>"AC9" As "¿Qué tan cumplida ha sido la Universidad Ean respecto a la promesa de valor académica ofrecida por el programa que cursas actualmente?",</t>
+  </si>
+  <si>
+    <t>"AC2" As "Competencias para la enseñanza y la formación",</t>
+  </si>
+  <si>
+    <t>NULL As "Cumplimiento del syllabus y plan de estudios del programa",</t>
+  </si>
+  <si>
+    <t>"AC4" As "Evaluación y acompañamiento del proceso de aprendizaje",</t>
+  </si>
+  <si>
+    <t>"AC5" As "Entrega de calificaciones y retroalimentación",</t>
+  </si>
+  <si>
+    <t>"AC3" As "Calidad humana",</t>
+  </si>
+  <si>
+    <t>NULL  As "Manejo tecnológico",</t>
+  </si>
+  <si>
+    <t>NULL  As "Decano(a)",</t>
+  </si>
+  <si>
+    <t>"AC7" As "Director(a) de Programa o Coordinador",</t>
+  </si>
+  <si>
+    <t>"AC10" As "Satisfacción entrega material VAC",</t>
+  </si>
+  <si>
+    <t>"AC8" As "Satisfacción asistentes facultad",</t>
+  </si>
+  <si>
+    <t>"AC11" As "Probabilidad recomendar programa académico",</t>
+  </si>
+  <si>
+    <t>NULL  As "Probabilidad volver a estudiar en EAN",</t>
+  </si>
+  <si>
+    <t>NULL  As "Cuerpo docente con experiencia profesional"</t>
   </si>
 </sst>
 </file>
@@ -692,5 +825,224 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="90" verticalDpi="90" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1C19BFC-0F7C-4F5B-BC52-76B23C6DFC86}">
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>64</v>
+      </c>
+      <c r="I6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="I7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="I8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="I9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="I11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="I12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>68</v>
+      </c>
+      <c r="I13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>70</v>
+      </c>
+      <c r="I15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>72</v>
+      </c>
+      <c r="I17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="I18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>73</v>
+      </c>
+      <c r="I19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>74</v>
+      </c>
+      <c r="I20" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>75</v>
+      </c>
+      <c r="I21" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>76</v>
+      </c>
+      <c r="I22" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>77</v>
+      </c>
+      <c r="I23" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>78</v>
+      </c>
+      <c r="I24" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>79</v>
+      </c>
+      <c r="I25" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>80</v>
+      </c>
+      <c r="I26" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>